<commit_message>
Add a count for the past year only
</commit_message>
<xml_diff>
--- a/rcc-song-summary/RCC Song List Template.xlsx
+++ b/rcc-song-summary/RCC Song List Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\drump\Code\rcc-utils\rcc-song-summary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B4184E5-782F-44B6-8AFC-BB77383F2548}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FDC4ECC-F30D-43C2-B0ED-47BF3C6EC01D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Song List" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Folder</t>
   </si>
@@ -48,6 +48,9 @@
   </si>
   <si>
     <t>Most Recent</t>
+  </si>
+  <si>
+    <t>Past Year</t>
   </si>
 </sst>
 </file>
@@ -460,19 +463,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="43" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="28.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="29.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.5703125" customWidth="1"/>
-    <col min="6" max="7" width="13.5703125" style="3" customWidth="1"/>
-    <col min="8" max="8" width="89.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="13.5703125" customWidth="1"/>
+    <col min="7" max="8" width="13.5703125" style="3" customWidth="1"/>
+    <col min="9" max="9" width="89.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -488,16 +491,19 @@
       <c r="E1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -513,7 +519,7 @@
       <formula>"Bethel"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E1:E1048576">
+  <conditionalFormatting sqref="E1:F1048576">
     <cfRule type="dataBar" priority="1">
       <dataBar>
         <cfvo type="min"/>
@@ -527,7 +533,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F1:F1048576">
+  <conditionalFormatting sqref="G1:G1048576">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -537,7 +543,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G1:G1048576">
+  <conditionalFormatting sqref="H1:H1048576">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -562,7 +568,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>E1:E1048576</xm:sqref>
+          <xm:sqref>E1:F1048576</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>

</xml_diff>

<commit_message>
Add a list of individual dates and leaders to the song list spreadsheet
</commit_message>
<xml_diff>
--- a/rcc-song-summary/RCC Song List Template.xlsx
+++ b/rcc-song-summary/RCC Song List Template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\drump\Code\rcc-utils\rcc-song-summary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FDC4ECC-F30D-43C2-B0ED-47BF3C6EC01D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22DC2B1B-3D65-4AC5-9784-06561D40F658}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Folder</t>
   </si>
@@ -51,6 +51,9 @@
   </si>
   <si>
     <t>Past Year</t>
+  </si>
+  <si>
+    <t>All Dates</t>
   </si>
 </sst>
 </file>
@@ -463,7 +466,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
@@ -475,7 +478,7 @@
     <col min="9" max="9" width="89.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -505,6 +508,9 @@
       </c>
       <c r="J1" s="1" t="s">
         <v>5</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>